<commit_message>
fix: standardize report header formatting
</commit_message>
<xml_diff>
--- a/public/templates/CITYBUS-BAO-CAO-GPS-BP-QLCL-DV.xlsx
+++ b/public/templates/CITYBUS-BAO-CAO-GPS-BP-QLCL-DV.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duykha/Downloads/qlcldv/public/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duykha/Workspace/reactjs/qlcldv/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4AD7EB-9730-CD44-A3EA-A1694105B631}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940DCDAF-A2AC-C846-B58E-D232FFD024B3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -257,7 +257,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -280,43 +280,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -326,7 +289,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -370,6 +333,15 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -379,34 +351,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -722,70 +670,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="3" spans="1:10" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
+      <c r="A3" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="1:10" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
       <c r="F4" s="22"/>
     </row>
     <row r="5" spans="1:10" s="1" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="27"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
     </row>
     <row r="6" spans="1:10" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
     </row>
     <row r="7" spans="1:10" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="2" t="s">
         <v>4</v>
       </c>
@@ -818,10 +766,10 @@
       </c>
     </row>
     <row r="9" spans="1:10" s="1" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="24"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="10">
         <f>SUM(C8:C8)</f>
         <v>0</v>
@@ -840,34 +788,34 @@
       </c>
     </row>
     <row r="10" spans="1:10" s="7" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" s="7" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" s="7" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="23"/>
-      <c r="B12" s="23"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="2" t="s">
         <v>4</v>
       </c>
@@ -901,10 +849,10 @@
       </c>
     </row>
     <row r="14" spans="1:10" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="24"/>
+      <c r="B14" s="17"/>
       <c r="C14" s="10">
         <f>SUM(C13)</f>
         <v>0</v>
@@ -924,32 +872,32 @@
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" s="1" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
     </row>
     <row r="16" spans="1:10" s="1" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
     </row>
     <row r="17" spans="1:6" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="2" t="s">
         <v>4</v>
       </c>
@@ -982,10 +930,10 @@
       </c>
     </row>
     <row r="19" spans="1:6" s="1" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="24"/>
+      <c r="B19" s="17"/>
       <c r="C19" s="10">
         <f>SUM(C18:C18)</f>
         <v>0</v>
@@ -1004,32 +952,32 @@
       </c>
     </row>
     <row r="20" spans="1:6" s="1" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
     </row>
     <row r="21" spans="1:6" s="1" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
     </row>
     <row r="22" spans="1:6" s="1" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
+      <c r="A22" s="16"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="2" t="s">
         <v>4</v>
       </c>
@@ -1062,10 +1010,10 @@
       </c>
     </row>
     <row r="24" spans="1:6" s="1" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="24" t="s">
+      <c r="A24" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="24"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="9">
         <f>SUM(C23)</f>
         <v>0</v>
@@ -1084,87 +1032,77 @@
       </c>
     </row>
     <row r="25" spans="1:6" s="1" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
     </row>
     <row r="26" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="16" t="s">
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
     </row>
     <row r="27" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="17"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
+      <c r="A27" s="20"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
     </row>
     <row r="28" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="17"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
     </row>
     <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="17"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
     </row>
     <row r="30" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="17"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
     </row>
     <row r="31" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="17"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
     </row>
     <row r="32" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="17"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A1:F2"/>
     <mergeCell ref="A26:C32"/>
     <mergeCell ref="D26:F32"/>
@@ -1181,6 +1119,16 @@
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:F6"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="A24:B24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>